<commit_message>
Replace property listings from updated spreadsheet
</commit_message>
<xml_diff>
--- a/data/AI-assistant.xlsx
+++ b/data/AI-assistant.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="8615"/>
+    <workbookView windowWidth="24750" windowHeight="12080"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="201">
   <si>
     <t>小区</t>
   </si>
@@ -98,7 +98,7 @@
     <t>⭐⭐⭐</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AvkBOWF56</t>
+    <t>https://weixin.qq.com/sph/AutNW8uDF</t>
   </si>
   <si>
     <t>望族新城</t>
@@ -125,7 +125,7 @@
     <t>⭐⭐⭐⭐</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AOCQGgox6</t>
+    <t>https://weixin.qq.com/sph/ACHgexhxS</t>
   </si>
   <si>
     <t>万源城尚郡</t>
@@ -149,7 +149,7 @@
     <t>楼王户型，2梯2户</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/A1tc1dAsx</t>
+    <t>https://weixin.qq.com/sph/A3b0riNEd</t>
   </si>
   <si>
     <t>融创玫瑰公馆</t>
@@ -170,7 +170,7 @@
     <t>次新品质小区、最低总价</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/ArstqH5Kd</t>
+    <t>https://weixin.qq.com/sph/AU2Qpld7G</t>
   </si>
   <si>
     <t>899万</t>
@@ -182,7 +182,7 @@
     <t>⭐⭐⭐⭐+</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AOBFho8un</t>
+    <t>https://weixin.qq.com/sph/Akasnr30K</t>
   </si>
   <si>
     <t>万源城御璄</t>
@@ -209,7 +209,7 @@
     <t>品质大平层，最低总价</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AgFOIvbbm</t>
+    <t>https://weixin.qq.com/sph/ATsrITLaW</t>
   </si>
   <si>
     <t>蔚蓝城市花园</t>
@@ -227,7 +227,7 @@
     <t>安静位置</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/APhhZgvTu</t>
+    <t>https://weixin.qq.com/sph/AXnWeoilQ</t>
   </si>
   <si>
     <t>新时代富嘉花园</t>
@@ -245,6 +245,9 @@
     <t>平吉小学、龙茗中学</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AqPkkwhId</t>
+  </si>
+  <si>
     <t>当代艺墅</t>
   </si>
   <si>
@@ -275,7 +278,7 @@
     <t>安静位置，二期翻新</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AdZNRwqVw</t>
+    <t>https://weixin.qq.com/sph/AT1S4qMcR</t>
   </si>
   <si>
     <t>264㎡</t>
@@ -293,7 +296,7 @@
     <t>内圈位置</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AvR3GWlm1</t>
+    <t>https://weixin.qq.com/sph/AYlW0mJ57</t>
   </si>
   <si>
     <t>万源城朗郡</t>
@@ -317,7 +320,7 @@
     <t>⭐⭐⭐+</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/A0L9PooRN</t>
+    <t>https://weixin.qq.com/sph/AdcCYcNOs</t>
   </si>
   <si>
     <t>新时代景庭</t>
@@ -332,7 +335,7 @@
     <t>环境优雅</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AnRtmdcvZ</t>
+    <t>https://weixin.qq.com/sph/AM4oYrEe2</t>
   </si>
   <si>
     <t>上海花园</t>
@@ -362,7 +365,7 @@
     <t>洋房外销房</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AnCbLG871</t>
+    <t>https://weixin.qq.com/sph/A0ewY1XT1</t>
   </si>
   <si>
     <t>122㎡</t>
@@ -413,7 +416,7 @@
     <t>北入户南花园，大独栋</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/A965QcM37</t>
+    <t>https://weixin.qq.com/sph/Aj996g6s2</t>
   </si>
   <si>
     <t>1730万</t>
@@ -434,7 +437,7 @@
     <t>人车分离小区，景观房</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AXJ97oZwb</t>
+    <t>https://weixin.qq.com/sph/ArCpUnix7</t>
   </si>
   <si>
     <t>221㎡</t>
@@ -455,9 +458,6 @@
     <t>人车分离，顶楼复式</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/ACxSJciOX</t>
-  </si>
-  <si>
     <t>1650万</t>
   </si>
   <si>
@@ -506,7 +506,7 @@
     <t>双南两房，可改三房</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AYVy1GV2C</t>
+    <t>https://weixin.qq.com/sph/AxDnZAY26</t>
   </si>
   <si>
     <t>142㎡</t>
@@ -594,6 +594,42 @@
   </si>
   <si>
     <t>次新品质小区</t>
+  </si>
+  <si>
+    <t>152㎡</t>
+  </si>
+  <si>
+    <t>1420万</t>
+  </si>
+  <si>
+    <t>绿化景观楼层位置</t>
+  </si>
+  <si>
+    <t>康健丽都</t>
+  </si>
+  <si>
+    <t>98㎡</t>
+  </si>
+  <si>
+    <t>698万</t>
+  </si>
+  <si>
+    <t>670万</t>
+  </si>
+  <si>
+    <t>边套户型，拐角大飘窗</t>
+  </si>
+  <si>
+    <t>136㎡</t>
+  </si>
+  <si>
+    <t>96㎡</t>
+  </si>
+  <si>
+    <t>1100万</t>
+  </si>
+  <si>
+    <t>次新品质小区，位置好</t>
   </si>
 </sst>
 </file>
@@ -1754,22 +1790,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M31"/>
-  <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4"/>
+  <dimension ref="A1:M35"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="14.9074074074074" customWidth="1"/>
-    <col min="2" max="2" width="8.63888888888889" customWidth="1"/>
+    <col min="1" max="1" width="14.9090909090909" customWidth="1"/>
+    <col min="2" max="2" width="8.63636363636364" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="7.73148148148148" customWidth="1"/>
-    <col min="5" max="5" width="7.4537037037037" customWidth="1"/>
-    <col min="6" max="6" width="6.63888888888889" customWidth="1"/>
-    <col min="7" max="7" width="19.0925925925926" customWidth="1"/>
-    <col min="8" max="8" width="11.1851851851852" customWidth="1"/>
-    <col min="9" max="9" width="8.81481481481481" customWidth="1"/>
-    <col min="10" max="10" width="9.81481481481481" customWidth="1"/>
-    <col min="11" max="11" width="23.8148148148148" customWidth="1"/>
+    <col min="4" max="4" width="7.72727272727273" customWidth="1"/>
+    <col min="5" max="5" width="7.45454545454545" customWidth="1"/>
+    <col min="6" max="6" width="6.63636363636364" customWidth="1"/>
+    <col min="7" max="7" width="19.0909090909091" customWidth="1"/>
+    <col min="8" max="8" width="11.1818181818182" customWidth="1"/>
+    <col min="9" max="9" width="8.81818181818182" customWidth="1"/>
+    <col min="10" max="10" width="9.81818181818182" customWidth="1"/>
+    <col min="11" max="11" width="23.8181818181818" customWidth="1"/>
     <col min="12" max="12" width="11" customWidth="1"/>
-    <col min="13" max="13" width="41.8148148148148" customWidth="1"/>
+    <col min="13" max="13" width="41.8181818181818" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -2138,48 +2174,48 @@
         <v>22</v>
       </c>
       <c r="M9" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J10" t="s">
         <v>38</v>
       </c>
       <c r="K10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="L10" t="s">
         <v>22</v>
       </c>
       <c r="M10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -2187,16 +2223,16 @@
         <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F11">
         <v>11</v>
@@ -2214,30 +2250,30 @@
         <v>58</v>
       </c>
       <c r="K11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L11" t="s">
         <v>31</v>
       </c>
       <c r="M11" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E12" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F12">
         <v>10</v>
@@ -2255,27 +2291,27 @@
         <v>38</v>
       </c>
       <c r="K12" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L12" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M12" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C13" t="s">
         <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E13" t="s">
         <v>70</v>
@@ -2296,39 +2332,39 @@
         <v>20</v>
       </c>
       <c r="K13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:13">
       <c r="A14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I14">
         <v>1993</v>
@@ -2337,27 +2373,27 @@
         <v>38</v>
       </c>
       <c r="K14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L14" t="s">
         <v>22</v>
       </c>
-      <c r="M14" t="s">
-        <v>111</v>
+      <c r="M14" s="2" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:13">
       <c r="A15" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E15" t="s">
         <v>27</v>
@@ -2378,12 +2414,12 @@
         <v>20</v>
       </c>
       <c r="K15" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="L15" t="s">
-        <v>95</v>
-      </c>
-      <c r="M15" t="s">
+        <v>96</v>
+      </c>
+      <c r="M15" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2392,16 +2428,16 @@
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F16">
         <v>12</v>
@@ -2419,7 +2455,7 @@
         <v>20</v>
       </c>
       <c r="K16" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="L16" t="s">
         <v>22</v>
@@ -2430,28 +2466,28 @@
     </row>
     <row r="17" spans="1:13">
       <c r="A17" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B17" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C17" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D17" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E17" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F17" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G17" t="s">
         <v>44</v>
       </c>
       <c r="H17" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I17">
         <v>2004</v>
@@ -2460,30 +2496,30 @@
         <v>20</v>
       </c>
       <c r="K17" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="L17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M17" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="1:13">
       <c r="A18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D18" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E18" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F18">
         <v>3</v>
@@ -2501,10 +2537,10 @@
         <v>38</v>
       </c>
       <c r="K18" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M18" t="s">
         <v>40</v>
@@ -2515,16 +2551,16 @@
         <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C19" t="s">
         <v>69</v>
       </c>
       <c r="D19" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E19" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F19">
         <v>9</v>
@@ -2542,13 +2578,13 @@
         <v>38</v>
       </c>
       <c r="K19" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L19" t="s">
         <v>22</v>
       </c>
       <c r="M19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -2556,16 +2592,16 @@
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C20" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D20" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E20" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F20">
         <v>15</v>
@@ -2580,27 +2616,27 @@
         <v>2008</v>
       </c>
       <c r="J20" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K20" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L20" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M20" t="s">
-        <v>142</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:13">
       <c r="A21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C21" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D21" t="s">
         <v>143</v>
@@ -2630,7 +2666,7 @@
         <v>50</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -2668,27 +2704,27 @@
         <v>150</v>
       </c>
       <c r="L22" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M22" t="s">
-        <v>40</v>
+        <v>129</v>
       </c>
     </row>
     <row r="23" spans="1:13">
       <c r="A23" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B23" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C23" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D23" t="s">
         <v>151</v>
       </c>
       <c r="E23" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F23">
         <v>6</v>
@@ -2717,13 +2753,13 @@
     </row>
     <row r="24" spans="1:13">
       <c r="A24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B24" t="s">
         <v>153</v>
       </c>
       <c r="C24" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D24" t="s">
         <v>154</v>
@@ -2750,21 +2786,21 @@
         <v>155</v>
       </c>
       <c r="L24" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M24" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="25" spans="1:13">
       <c r="A25" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B25" t="s">
         <v>156</v>
       </c>
       <c r="C25" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D25" t="s">
         <v>157</v>
@@ -2835,12 +2871,12 @@
         <v>22</v>
       </c>
       <c r="M26" t="s">
-        <v>142</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:13">
       <c r="A27" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B27" t="s">
         <v>164</v>
@@ -2876,7 +2912,7 @@
         <v>31</v>
       </c>
       <c r="M27" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -2887,7 +2923,7 @@
         <v>171</v>
       </c>
       <c r="C28" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D28" t="s">
         <v>172</v>
@@ -2914,10 +2950,10 @@
         <v>175</v>
       </c>
       <c r="L28" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M28" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -2958,12 +2994,12 @@
         <v>31</v>
       </c>
       <c r="M29" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="30" spans="1:13">
       <c r="A30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B30" t="s">
         <v>180</v>
@@ -2998,8 +3034,8 @@
       <c r="L30" t="s">
         <v>31</v>
       </c>
-      <c r="M30" t="s">
-        <v>111</v>
+      <c r="M30" s="2" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="31" spans="1:13">
@@ -3016,7 +3052,7 @@
         <v>187</v>
       </c>
       <c r="E31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F31">
         <v>10</v>
@@ -3039,16 +3075,178 @@
       <c r="L31" t="s">
         <v>22</v>
       </c>
-      <c r="M31" s="2" t="s">
-        <v>128</v>
+      <c r="M31" s="3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13">
+      <c r="A32" t="s">
+        <v>90</v>
+      </c>
+      <c r="B32" t="s">
+        <v>189</v>
+      </c>
+      <c r="C32" t="s">
+        <v>15</v>
+      </c>
+      <c r="D32" t="s">
+        <v>190</v>
+      </c>
+      <c r="E32" t="s">
+        <v>162</v>
+      </c>
+      <c r="F32">
+        <v>7</v>
+      </c>
+      <c r="G32" t="s">
+        <v>18</v>
+      </c>
+      <c r="H32" t="s">
+        <v>19</v>
+      </c>
+      <c r="I32">
+        <v>2010</v>
+      </c>
+      <c r="J32" t="s">
+        <v>20</v>
+      </c>
+      <c r="K32" t="s">
+        <v>191</v>
+      </c>
+      <c r="L32" t="s">
+        <v>96</v>
+      </c>
+      <c r="M32" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13">
+      <c r="A33" t="s">
+        <v>192</v>
+      </c>
+      <c r="B33" t="s">
+        <v>193</v>
+      </c>
+      <c r="C33" t="s">
+        <v>69</v>
+      </c>
+      <c r="D33" t="s">
+        <v>194</v>
+      </c>
+      <c r="E33" t="s">
+        <v>195</v>
+      </c>
+      <c r="F33">
+        <v>12</v>
+      </c>
+      <c r="G33" t="s">
+        <v>28</v>
+      </c>
+      <c r="H33" t="s">
+        <v>45</v>
+      </c>
+      <c r="I33">
+        <v>2003</v>
+      </c>
+      <c r="J33" t="s">
+        <v>29</v>
+      </c>
+      <c r="K33" t="s">
+        <v>196</v>
+      </c>
+      <c r="L33" t="s">
+        <v>31</v>
+      </c>
+      <c r="M33" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13">
+      <c r="A34" t="s">
+        <v>192</v>
+      </c>
+      <c r="B34" t="s">
+        <v>197</v>
+      </c>
+      <c r="C34" t="s">
+        <v>15</v>
+      </c>
+      <c r="D34" t="s">
+        <v>36</v>
+      </c>
+      <c r="E34" t="s">
+        <v>37</v>
+      </c>
+      <c r="F34">
+        <v>4</v>
+      </c>
+      <c r="G34" t="s">
+        <v>28</v>
+      </c>
+      <c r="H34" t="s">
+        <v>45</v>
+      </c>
+      <c r="I34">
+        <v>2003</v>
+      </c>
+      <c r="J34" t="s">
+        <v>29</v>
+      </c>
+      <c r="K34" t="s">
+        <v>39</v>
+      </c>
+      <c r="L34" t="s">
+        <v>96</v>
+      </c>
+      <c r="M34" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13">
+      <c r="A35" t="s">
+        <v>41</v>
+      </c>
+      <c r="B35" t="s">
+        <v>198</v>
+      </c>
+      <c r="C35" t="s">
+        <v>35</v>
+      </c>
+      <c r="D35" t="s">
+        <v>199</v>
+      </c>
+      <c r="E35" t="s">
+        <v>27</v>
+      </c>
+      <c r="F35">
+        <v>5</v>
+      </c>
+      <c r="G35" t="s">
+        <v>44</v>
+      </c>
+      <c r="H35" t="s">
+        <v>45</v>
+      </c>
+      <c r="I35">
+        <v>2017</v>
+      </c>
+      <c r="J35" t="s">
+        <v>38</v>
+      </c>
+      <c r="K35" t="s">
+        <v>200</v>
+      </c>
+      <c r="L35" t="s">
+        <v>50</v>
+      </c>
+      <c r="M35" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="L2" r:id="rId1" display="⭐⭐⭐"/>
-    <hyperlink ref="M2" r:id="rId2" display="https://weixin.qq.com/sph/AvkBOWF56"/>
-    <hyperlink ref="M21" r:id="rId3" display="https://weixin.qq.com/sph/A0L9PooRN"/>
-    <hyperlink ref="M31" r:id="rId4" display="https://weixin.qq.com/sph/A965QcM37"/>
+    <hyperlink ref="M15" r:id="rId2" display="https://weixin.qq.com/sph/AutNW8uDF"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Replace listings with AI assistant 3 source
</commit_message>
<xml_diff>
--- a/data/AI-assistant.xlsx
+++ b/data/AI-assistant.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="225">
   <si>
     <t>小区</t>
   </si>
@@ -98,7 +98,7 @@
     <t>⭐⭐⭐</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AutNW8uDF</t>
+    <t>https://weixin.qq.com/sph/AWlVgciU0F</t>
   </si>
   <si>
     <t>望族新城</t>
@@ -125,7 +125,7 @@
     <t>⭐⭐⭐⭐</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/ACHgexhxS</t>
+    <t>https://weixin.qq.com/sph/A5GgyC2YOV</t>
   </si>
   <si>
     <t>万源城尚郡</t>
@@ -149,7 +149,7 @@
     <t>楼王户型，2梯2户</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/A3b0riNEd</t>
+    <t>https://weixin.qq.com/sph/AJhZ4fsxCd</t>
   </si>
   <si>
     <t>融创玫瑰公馆</t>
@@ -170,7 +170,7 @@
     <t>次新品质小区、最低总价</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AU2Qpld7G</t>
+    <t>https://weixin.qq.com/sph/ABHKnlbjpJ</t>
   </si>
   <si>
     <t>899万</t>
@@ -182,7 +182,7 @@
     <t>⭐⭐⭐⭐+</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/Akasnr30K</t>
+    <t>https://weixin.qq.com/sph/AAzm1sWE0I</t>
   </si>
   <si>
     <t>万源城御璄</t>
@@ -209,7 +209,7 @@
     <t>品质大平层，最低总价</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/ATsrITLaW</t>
+    <t>https://weixin.qq.com/sph/AVDJeMTwB2</t>
   </si>
   <si>
     <t>蔚蓝城市花园</t>
@@ -227,7 +227,7 @@
     <t>安静位置</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AXnWeoilQ</t>
+    <t>https://weixin.qq.com/sph/AsdRcqEKQy</t>
   </si>
   <si>
     <t>新时代富嘉花园</t>
@@ -245,7 +245,7 @@
     <t>平吉小学、龙茗中学</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AqPkkwhId</t>
+    <t>https://weixin.qq.com/sph/AroQTC9mgT</t>
   </si>
   <si>
     <t>当代艺墅</t>
@@ -278,7 +278,7 @@
     <t>安静位置，二期翻新</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AT1S4qMcR</t>
+    <t>https://weixin.qq.com/sph/Al85SP0EM5</t>
   </si>
   <si>
     <t>264㎡</t>
@@ -296,7 +296,7 @@
     <t>内圈位置</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AYlW0mJ57</t>
+    <t>https://weixin.qq.com/sph/AatUqcql5O</t>
   </si>
   <si>
     <t>万源城朗郡</t>
@@ -320,7 +320,7 @@
     <t>⭐⭐⭐+</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AdcCYcNOs</t>
+    <t>https://weixin.qq.com/sph/AuYeL0SUC7</t>
   </si>
   <si>
     <t>新时代景庭</t>
@@ -335,7 +335,7 @@
     <t>环境优雅</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AM4oYrEe2</t>
+    <t>https://weixin.qq.com/sph/AjeJPotcni</t>
   </si>
   <si>
     <t>上海花园</t>
@@ -365,7 +365,7 @@
     <t>洋房外销房</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/A0ewY1XT1</t>
+    <t>https://weixin.qq.com/sph/AD7hUapFGV</t>
   </si>
   <si>
     <t>122㎡</t>
@@ -380,6 +380,9 @@
     <t>位置安静</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AMMld2Ec9u</t>
+  </si>
+  <si>
     <t>171㎡</t>
   </si>
   <si>
@@ -392,6 +395,9 @@
     <t>元宝户型，人车分离</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/A2QttHBtlj</t>
+  </si>
+  <si>
     <t>东苑古龙城</t>
   </si>
   <si>
@@ -416,7 +422,7 @@
     <t>北入户南花园，大独栋</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/Aj996g6s2</t>
+    <t>https://weixin.qq.com/sph/A7XGKfTf1z</t>
   </si>
   <si>
     <t>1730万</t>
@@ -425,6 +431,9 @@
     <t>1670万</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AcxGPIkz2S</t>
+  </si>
+  <si>
     <t>100㎡</t>
   </si>
   <si>
@@ -437,7 +446,7 @@
     <t>人车分离小区，景观房</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/ArCpUnix7</t>
+    <t>https://weixin.qq.com/sph/A0PR6wYw92</t>
   </si>
   <si>
     <t>221㎡</t>
@@ -458,6 +467,9 @@
     <t>人车分离，顶楼复式</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AcX434kuOb</t>
+  </si>
+  <si>
     <t>1650万</t>
   </si>
   <si>
@@ -467,6 +479,9 @@
     <t>小区性价比最高4房</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AHWgvan6PH</t>
+  </si>
+  <si>
     <t>297㎡</t>
   </si>
   <si>
@@ -482,12 +497,18 @@
     <t>品质大平层，带保姆房</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/Ap1V0RL6Qy</t>
+  </si>
+  <si>
     <t>1850万</t>
   </si>
   <si>
     <t>带入户花园</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AUKqQCblld</t>
+  </si>
+  <si>
     <t>115㎡</t>
   </si>
   <si>
@@ -497,6 +518,9 @@
     <t>双南两房，拎包入住</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AoufetHCGs</t>
+  </si>
+  <si>
     <t>121㎡</t>
   </si>
   <si>
@@ -506,7 +530,7 @@
     <t>双南两房，可改三房</t>
   </si>
   <si>
-    <t>https://weixin.qq.com/sph/AxDnZAY26</t>
+    <t>https://weixin.qq.com/sph/AwVjXRuo8j</t>
   </si>
   <si>
     <t>142㎡</t>
@@ -521,6 +545,9 @@
     <t>人车分离，高区景观房</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/ABerfPckO1</t>
+  </si>
+  <si>
     <t>249㎡</t>
   </si>
   <si>
@@ -542,6 +569,9 @@
     <t>小区最好的一套房源</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AijKOEHmGq</t>
+  </si>
+  <si>
     <t>144㎡</t>
   </si>
   <si>
@@ -557,6 +587,9 @@
     <t>景观房，拎包入住</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AN92juSpal</t>
+  </si>
+  <si>
     <t>世纪古美</t>
   </si>
   <si>
@@ -569,6 +602,9 @@
     <t>刚满五年次新小区</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/ApKy5f1P68</t>
+  </si>
+  <si>
     <t>148㎡</t>
   </si>
   <si>
@@ -587,6 +623,9 @@
     <t>可改4房，位置安静</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AwV2BNLagj</t>
+  </si>
+  <si>
     <t>123㎡</t>
   </si>
   <si>
@@ -596,6 +635,9 @@
     <t>次新品质小区</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AHQDm7VHNg</t>
+  </si>
+  <si>
     <t>152㎡</t>
   </si>
   <si>
@@ -605,6 +647,9 @@
     <t>绿化景观楼层位置</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AG0rWxLcSt</t>
+  </si>
+  <si>
     <t>康健丽都</t>
   </si>
   <si>
@@ -620,9 +665,15 @@
     <t>边套户型，拐角大飘窗</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AFzpUXkQh5</t>
+  </si>
+  <si>
     <t>136㎡</t>
   </si>
   <si>
+    <t>https://weixin.qq.com/sph/AHA8FUpaG4</t>
+  </si>
+  <si>
     <t>96㎡</t>
   </si>
   <si>
@@ -630,6 +681,27 @@
   </si>
   <si>
     <t>次新品质小区，位置好</t>
+  </si>
+  <si>
+    <t>https://weixin.qq.com/sph/AzuJSX02AY</t>
+  </si>
+  <si>
+    <t>162㎡</t>
+  </si>
+  <si>
+    <t>1400万</t>
+  </si>
+  <si>
+    <t>顶楼复式，大露台</t>
+  </si>
+  <si>
+    <t>https://weixin.qq.com/sph/Aglh2wqd6a</t>
+  </si>
+  <si>
+    <t>电梯洋房</t>
+  </si>
+  <si>
+    <t>https://weixin.qq.com/sph/ApLRHE1Mf5</t>
   </si>
 </sst>
 </file>
@@ -1790,7 +1862,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="14.9090909090909" customWidth="1"/>
@@ -1927,7 +1999,7 @@
       <c r="L3" t="s">
         <v>31</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="M3" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2009,7 +2081,7 @@
       <c r="L5" t="s">
         <v>31</v>
       </c>
-      <c r="M5" t="s">
+      <c r="M5" s="2" t="s">
         <v>47</v>
       </c>
     </row>
@@ -2050,7 +2122,7 @@
       <c r="L6" t="s">
         <v>50</v>
       </c>
-      <c r="M6" t="s">
+      <c r="M6" s="2" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2091,7 +2163,7 @@
       <c r="L7" t="s">
         <v>50</v>
       </c>
-      <c r="M7" t="s">
+      <c r="M7" s="2" t="s">
         <v>60</v>
       </c>
     </row>
@@ -2132,7 +2204,7 @@
       <c r="L8" t="s">
         <v>22</v>
       </c>
-      <c r="M8" t="s">
+      <c r="M8" s="2" t="s">
         <v>66</v>
       </c>
     </row>
@@ -2173,7 +2245,7 @@
       <c r="L9" t="s">
         <v>22</v>
       </c>
-      <c r="M9" t="s">
+      <c r="M9" s="2" t="s">
         <v>72</v>
       </c>
     </row>
@@ -2214,7 +2286,7 @@
       <c r="L10" t="s">
         <v>22</v>
       </c>
-      <c r="M10" t="s">
+      <c r="M10" s="3" t="s">
         <v>83</v>
       </c>
     </row>
@@ -2255,7 +2327,7 @@
       <c r="L11" t="s">
         <v>31</v>
       </c>
-      <c r="M11" t="s">
+      <c r="M11" s="3" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2296,7 +2368,7 @@
       <c r="L12" t="s">
         <v>96</v>
       </c>
-      <c r="M12" t="s">
+      <c r="M12" s="2" t="s">
         <v>97</v>
       </c>
     </row>
@@ -2337,7 +2409,7 @@
       <c r="L13" t="s">
         <v>96</v>
       </c>
-      <c r="M13" t="s">
+      <c r="M13" s="2" t="s">
         <v>102</v>
       </c>
     </row>
@@ -2420,7 +2492,7 @@
         <v>96</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>23</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -2428,16 +2500,16 @@
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C16" t="s">
         <v>92</v>
       </c>
       <c r="D16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E16" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F16">
         <v>12</v>
@@ -2455,39 +2527,39 @@
         <v>20</v>
       </c>
       <c r="K16" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L16" t="s">
         <v>22</v>
       </c>
-      <c r="M16" t="s">
-        <v>32</v>
+      <c r="M16" s="2" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:13">
       <c r="A17" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B17" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C17" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D17" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E17" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F17" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G17" t="s">
         <v>44</v>
       </c>
       <c r="H17" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I17">
         <v>2004</v>
@@ -2496,13 +2568,13 @@
         <v>20</v>
       </c>
       <c r="K17" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="L17" t="s">
         <v>96</v>
       </c>
-      <c r="M17" t="s">
-        <v>129</v>
+      <c r="M17" s="2" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -2516,10 +2588,10 @@
         <v>92</v>
       </c>
       <c r="D18" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E18" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F18">
         <v>3</v>
@@ -2542,8 +2614,8 @@
       <c r="L18" t="s">
         <v>96</v>
       </c>
-      <c r="M18" t="s">
-        <v>40</v>
+      <c r="M18" s="2" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -2551,16 +2623,16 @@
         <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C19" t="s">
         <v>69</v>
       </c>
       <c r="D19" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E19" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F19">
         <v>9</v>
@@ -2578,13 +2650,13 @@
         <v>38</v>
       </c>
       <c r="K19" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="L19" t="s">
         <v>22</v>
       </c>
-      <c r="M19" t="s">
-        <v>136</v>
+      <c r="M19" s="2" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -2592,16 +2664,16 @@
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C20" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="D20" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="E20" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="F20">
         <v>15</v>
@@ -2616,16 +2688,16 @@
         <v>2008</v>
       </c>
       <c r="J20" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="K20" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="L20" t="s">
         <v>96</v>
       </c>
-      <c r="M20" t="s">
-        <v>66</v>
+      <c r="M20" s="2" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -2633,16 +2705,16 @@
         <v>90</v>
       </c>
       <c r="B21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C21" t="s">
         <v>92</v>
       </c>
       <c r="D21" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="E21" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="F21">
         <v>14</v>
@@ -2660,13 +2732,13 @@
         <v>20</v>
       </c>
       <c r="K21" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="L21" t="s">
         <v>50</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>97</v>
+        <v>150</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -2674,16 +2746,16 @@
         <v>52</v>
       </c>
       <c r="B22" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C22" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="D22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="E22" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="F22">
         <v>8</v>
@@ -2701,13 +2773,13 @@
         <v>58</v>
       </c>
       <c r="K22" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="L22" t="s">
         <v>96</v>
       </c>
       <c r="M22" t="s">
-        <v>129</v>
+        <v>156</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -2721,7 +2793,7 @@
         <v>92</v>
       </c>
       <c r="D23" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="E23" t="s">
         <v>94</v>
@@ -2742,13 +2814,13 @@
         <v>20</v>
       </c>
       <c r="K23" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="L23" t="s">
         <v>22</v>
       </c>
-      <c r="M23" t="s">
-        <v>51</v>
+      <c r="M23" s="2" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -2756,13 +2828,13 @@
         <v>90</v>
       </c>
       <c r="B24" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="C24" t="s">
         <v>114</v>
       </c>
       <c r="D24" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="E24" t="s">
         <v>27</v>
@@ -2783,13 +2855,13 @@
         <v>38</v>
       </c>
       <c r="K24" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="L24" t="s">
         <v>96</v>
       </c>
-      <c r="M24" t="s">
-        <v>136</v>
+      <c r="M24" s="2" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -2797,13 +2869,13 @@
         <v>90</v>
       </c>
       <c r="B25" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="C25" t="s">
         <v>114</v>
       </c>
       <c r="D25" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="E25" t="s">
         <v>26</v>
@@ -2824,13 +2896,13 @@
         <v>20</v>
       </c>
       <c r="K25" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="L25" t="s">
         <v>22</v>
       </c>
-      <c r="M25" t="s">
-        <v>159</v>
+      <c r="M25" s="2" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -2838,16 +2910,16 @@
         <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="C26" t="s">
         <v>15</v>
       </c>
       <c r="D26" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="E26" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="F26">
         <v>14</v>
@@ -2865,13 +2937,13 @@
         <v>20</v>
       </c>
       <c r="K26" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="L26" t="s">
         <v>22</v>
       </c>
-      <c r="M26" t="s">
-        <v>66</v>
+      <c r="M26" s="2" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -2879,25 +2951,25 @@
         <v>98</v>
       </c>
       <c r="B27" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="C27" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="D27" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="E27" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="F27" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="G27" t="s">
         <v>44</v>
       </c>
       <c r="H27" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="I27">
         <v>2004</v>
@@ -2906,13 +2978,13 @@
         <v>20</v>
       </c>
       <c r="K27" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="L27" t="s">
         <v>31</v>
       </c>
-      <c r="M27" t="s">
-        <v>83</v>
+      <c r="M27" s="2" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -2920,16 +2992,16 @@
         <v>41</v>
       </c>
       <c r="B28" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="C28" t="s">
         <v>92</v>
       </c>
       <c r="D28" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="E28" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="F28">
         <v>6</v>
@@ -2938,7 +3010,7 @@
         <v>44</v>
       </c>
       <c r="H28" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="I28">
         <v>2017</v>
@@ -2947,18 +3019,18 @@
         <v>38</v>
       </c>
       <c r="K28" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="L28" t="s">
         <v>96</v>
       </c>
-      <c r="M28" t="s">
-        <v>97</v>
+      <c r="M28" s="2" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="29" spans="1:13">
       <c r="A29" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="B29" t="s">
         <v>42</v>
@@ -2967,7 +3039,7 @@
         <v>15</v>
       </c>
       <c r="D29" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="E29" t="s">
         <v>36</v>
@@ -2976,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="G29" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="H29" t="s">
         <v>45</v>
@@ -2988,13 +3060,13 @@
         <v>38</v>
       </c>
       <c r="K29" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="L29" t="s">
         <v>31</v>
       </c>
-      <c r="M29" t="s">
-        <v>129</v>
+      <c r="M29" s="2" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -3002,16 +3074,16 @@
         <v>98</v>
       </c>
       <c r="B30" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="C30" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="D30" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="E30" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="F30">
         <v>4</v>
@@ -3026,16 +3098,16 @@
         <v>2004</v>
       </c>
       <c r="J30" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="K30" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="L30" t="s">
         <v>31</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>112</v>
+        <v>198</v>
       </c>
     </row>
     <row r="31" spans="1:13">
@@ -3043,13 +3115,13 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="C31" t="s">
         <v>15</v>
       </c>
       <c r="D31" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="E31" t="s">
         <v>106</v>
@@ -3070,13 +3142,13 @@
         <v>38</v>
       </c>
       <c r="K31" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="L31" t="s">
         <v>22</v>
       </c>
-      <c r="M31" s="3" t="s">
-        <v>129</v>
+      <c r="M31" s="2" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -3084,16 +3156,16 @@
         <v>90</v>
       </c>
       <c r="B32" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="C32" t="s">
         <v>15</v>
       </c>
       <c r="D32" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="E32" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="F32">
         <v>7</v>
@@ -3111,30 +3183,30 @@
         <v>20</v>
       </c>
       <c r="K32" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
       <c r="L32" t="s">
         <v>96</v>
       </c>
-      <c r="M32" t="s">
-        <v>102</v>
+      <c r="M32" s="2" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="33" spans="1:13">
       <c r="A33" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="B33" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="C33" t="s">
         <v>69</v>
       </c>
       <c r="D33" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="E33" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="F33">
         <v>12</v>
@@ -3152,21 +3224,21 @@
         <v>29</v>
       </c>
       <c r="K33" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
       <c r="L33" t="s">
         <v>31</v>
       </c>
-      <c r="M33" t="s">
-        <v>97</v>
+      <c r="M33" s="2" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="34" spans="1:13">
       <c r="A34" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="B34" t="s">
-        <v>197</v>
+        <v>213</v>
       </c>
       <c r="C34" t="s">
         <v>15</v>
@@ -3198,8 +3270,8 @@
       <c r="L34" t="s">
         <v>96</v>
       </c>
-      <c r="M34" t="s">
-        <v>83</v>
+      <c r="M34" s="2" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -3207,13 +3279,13 @@
         <v>41</v>
       </c>
       <c r="B35" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="C35" t="s">
         <v>35</v>
       </c>
       <c r="D35" t="s">
-        <v>199</v>
+        <v>216</v>
       </c>
       <c r="E35" t="s">
         <v>27</v>
@@ -3234,19 +3306,132 @@
         <v>38</v>
       </c>
       <c r="K35" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="L35" t="s">
         <v>50</v>
       </c>
-      <c r="M35" t="s">
-        <v>89</v>
+      <c r="M35" s="2" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13">
+      <c r="A36" t="s">
+        <v>67</v>
+      </c>
+      <c r="B36" t="s">
+        <v>219</v>
+      </c>
+      <c r="C36" t="s">
+        <v>85</v>
+      </c>
+      <c r="D36" t="s">
+        <v>200</v>
+      </c>
+      <c r="E36" t="s">
+        <v>220</v>
+      </c>
+      <c r="F36">
+        <v>11</v>
+      </c>
+      <c r="G36" t="s">
+        <v>71</v>
+      </c>
+      <c r="H36" t="s">
+        <v>45</v>
+      </c>
+      <c r="I36">
+        <v>2007</v>
+      </c>
+      <c r="J36" t="s">
+        <v>38</v>
+      </c>
+      <c r="K36" t="s">
+        <v>221</v>
+      </c>
+      <c r="L36" t="s">
+        <v>22</v>
+      </c>
+      <c r="M36" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
+      <c r="A37" t="s">
+        <v>123</v>
+      </c>
+      <c r="B37" t="s">
+        <v>219</v>
+      </c>
+      <c r="C37" t="s">
+        <v>92</v>
+      </c>
+      <c r="D37" t="s">
+        <v>220</v>
+      </c>
+      <c r="E37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37">
+        <v>3</v>
+      </c>
+      <c r="G37" t="s">
+        <v>44</v>
+      </c>
+      <c r="H37" t="s">
+        <v>45</v>
+      </c>
+      <c r="I37">
+        <v>2004</v>
+      </c>
+      <c r="J37" t="s">
+        <v>29</v>
+      </c>
+      <c r="K37" t="s">
+        <v>223</v>
+      </c>
+      <c r="L37" t="s">
+        <v>22</v>
+      </c>
+      <c r="M37" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="L2" r:id="rId1" display="⭐⭐⭐"/>
-    <hyperlink ref="M15" r:id="rId2" display="https://weixin.qq.com/sph/AutNW8uDF"/>
+    <hyperlink ref="M15" r:id="rId2" display="https://weixin.qq.com/sph/AMMld2Ec9u" tooltip="https://weixin.qq.com/sph/AMMld2Ec9u"/>
+    <hyperlink ref="M5" r:id="rId3" display="https://weixin.qq.com/sph/ABHKnlbjpJ" tooltip="https://weixin.qq.com/sph/ABHKnlbjpJ"/>
+    <hyperlink ref="M10" r:id="rId4" display="https://weixin.qq.com/sph/Al85SP0EM5" tooltip="https://weixin.qq.com/sph/Al85SP0EM5"/>
+    <hyperlink ref="M11" r:id="rId5" display="https://weixin.qq.com/sph/AatUqcql5O" tooltip="https://weixin.qq.com/sph/AatUqcql5O"/>
+    <hyperlink ref="M33" r:id="rId6" display="https://weixin.qq.com/sph/AFzpUXkQh5"/>
+    <hyperlink ref="M34" r:id="rId7" display="https://weixin.qq.com/sph/AHA8FUpaG4"/>
+    <hyperlink ref="M35" r:id="rId8" display="https://weixin.qq.com/sph/AzuJSX02AY"/>
+    <hyperlink ref="M32" r:id="rId9" display="https://weixin.qq.com/sph/AG0rWxLcSt"/>
+    <hyperlink ref="M30" r:id="rId10" display="https://weixin.qq.com/sph/AwV2BNLagj"/>
+    <hyperlink ref="M31" r:id="rId11" display="https://weixin.qq.com/sph/AHQDm7VHNg"/>
+    <hyperlink ref="M2" r:id="rId12" display="https://weixin.qq.com/sph/AWlVgciU0F"/>
+    <hyperlink ref="M3" r:id="rId13" display="https://weixin.qq.com/sph/A5GgyC2YOV"/>
+    <hyperlink ref="M6" r:id="rId14" display="https://weixin.qq.com/sph/AAzm1sWE0I" tooltip="https://weixin.qq.com/sph/AAzm1sWE0I"/>
+    <hyperlink ref="M7" r:id="rId15" display="https://weixin.qq.com/sph/AVDJeMTwB2"/>
+    <hyperlink ref="M8" r:id="rId16" display="https://weixin.qq.com/sph/AsdRcqEKQy"/>
+    <hyperlink ref="M9" r:id="rId17" display="https://weixin.qq.com/sph/AroQTC9mgT"/>
+    <hyperlink ref="M12" r:id="rId18" display="https://weixin.qq.com/sph/AuYeL0SUC7"/>
+    <hyperlink ref="M13" r:id="rId19" display="https://weixin.qq.com/sph/AjeJPotcni"/>
+    <hyperlink ref="M14" r:id="rId20" display="https://weixin.qq.com/sph/AD7hUapFGV"/>
+    <hyperlink ref="M16" r:id="rId21" display="https://weixin.qq.com/sph/A2QttHBtlj"/>
+    <hyperlink ref="M17" r:id="rId22" display="https://weixin.qq.com/sph/A7XGKfTf1z"/>
+    <hyperlink ref="M18" r:id="rId23" display="https://weixin.qq.com/sph/AcxGPIkz2S"/>
+    <hyperlink ref="M19" r:id="rId24" display="https://weixin.qq.com/sph/A0PR6wYw92"/>
+    <hyperlink ref="M20" r:id="rId25" display="https://weixin.qq.com/sph/AcX434kuOb"/>
+    <hyperlink ref="M21" r:id="rId26" display="https://weixin.qq.com/sph/AHWgvan6PH"/>
+    <hyperlink ref="M23" r:id="rId27" display="https://weixin.qq.com/sph/AUKqQCblld"/>
+    <hyperlink ref="M24" r:id="rId28" display="https://weixin.qq.com/sph/AoufetHCGs"/>
+    <hyperlink ref="M25" r:id="rId29" display="https://weixin.qq.com/sph/AwVjXRuo8j"/>
+    <hyperlink ref="M26" r:id="rId30" display="https://weixin.qq.com/sph/ABerfPckO1"/>
+    <hyperlink ref="M27" r:id="rId31" display="https://weixin.qq.com/sph/AijKOEHmGq"/>
+    <hyperlink ref="M28" r:id="rId32" display="https://weixin.qq.com/sph/AN92juSpal"/>
+    <hyperlink ref="M29" r:id="rId33" display="https://weixin.qq.com/sph/ApKy5f1P68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>